<commit_message>
feat: updates on postman collection and test cases
</commit_message>
<xml_diff>
--- a/RESTful-booker-service-api.xlsx
+++ b/RESTful-booker-service-api.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="269">
   <si>
     <t>HIGH</t>
   </si>
@@ -816,9 +816,6 @@
     <t>TC_FT_BOOKING_054</t>
   </si>
   <si>
-    <t>1. Valid date format CCYY-MM-DD should be supported</t>
-  </si>
-  <si>
     <t>Response with new booking with nullable property "additionalneeds" and OK [200] status</t>
   </si>
   <si>
@@ -836,6 +833,12 @@
   <si>
     <t>1. User should provide valid access token
 2. A deleted booking with non-numeric ID should not exist</t>
+  </si>
+  <si>
+    <t>1. Only valid date format 'CCYY-MM-DD' should be supported</t>
+  </si>
+  <si>
+    <t>1. Only valid date with format 'CCYY-MM-DD' should be supported</t>
   </si>
 </sst>
 </file>
@@ -1134,7 +1137,177 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="241">
+  <dxfs count="128">
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="0"/>
@@ -1171,6 +1344,196 @@
       </font>
       <fill>
         <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor theme="4" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
@@ -1181,12 +1544,292 @@
       </font>
       <fill>
         <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor theme="7" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color auto="1"/>
       </font>
       <fill>
@@ -1337,7 +1980,77 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
       </font>
       <fill>
         <patternFill>
@@ -1347,10 +2060,40 @@
     </dxf>
     <dxf>
       <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="0"/>
       </font>
       <fill>
         <patternFill>
+          <bgColor theme="3" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor theme="4" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
@@ -1432,1876 +2175,6 @@
       <fill>
         <patternFill>
           <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3902,19 +2775,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RESTful_booker_service_api_v1_0_0" displayName="RESTful_booker_service_api_v1_0_0" ref="A1:K63" headerRowCount="0" totalsRowShown="0" headerRowDxfId="240" dataDxfId="239" tableBorderDxfId="238" totalsRowBorderDxfId="237">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RESTful_booker_service_api_v1_0_0" displayName="RESTful_booker_service_api_v1_0_0" ref="A1:K63" headerRowCount="0" totalsRowShown="0" headerRowDxfId="127" dataDxfId="126" tableBorderDxfId="125" totalsRowBorderDxfId="124">
   <tableColumns count="11">
-    <tableColumn id="12" name="Column12" headerRowDxfId="236" dataDxfId="235"/>
-    <tableColumn id="1" name="Column1" headerRowDxfId="234" dataDxfId="233"/>
-    <tableColumn id="3" name="Column4" headerRowDxfId="232" dataDxfId="231"/>
-    <tableColumn id="2" name="Column3" headerRowDxfId="230" dataDxfId="229"/>
-    <tableColumn id="4" name="Column5" headerRowDxfId="228" dataDxfId="227"/>
-    <tableColumn id="5" name="Column6" headerRowDxfId="226" dataDxfId="225"/>
-    <tableColumn id="13" name="Column2" headerRowDxfId="224"/>
-    <tableColumn id="14" name="Column11" headerRowDxfId="223"/>
-    <tableColumn id="6" name="Column7" headerRowDxfId="222" dataDxfId="221"/>
-    <tableColumn id="7" name="Column8" headerRowDxfId="220" dataDxfId="219"/>
-    <tableColumn id="9" name="Column10" headerRowDxfId="218" dataDxfId="217"/>
+    <tableColumn id="12" name="Column12" headerRowDxfId="123" dataDxfId="122"/>
+    <tableColumn id="1" name="Column1" headerRowDxfId="121" dataDxfId="120"/>
+    <tableColumn id="3" name="Column4" headerRowDxfId="119" dataDxfId="118"/>
+    <tableColumn id="2" name="Column3" headerRowDxfId="117" dataDxfId="116"/>
+    <tableColumn id="4" name="Column5" headerRowDxfId="115" dataDxfId="114"/>
+    <tableColumn id="5" name="Column6" headerRowDxfId="113" dataDxfId="112"/>
+    <tableColumn id="13" name="Column2" headerRowDxfId="111"/>
+    <tableColumn id="14" name="Column11" headerRowDxfId="110"/>
+    <tableColumn id="6" name="Column7" headerRowDxfId="109" dataDxfId="108"/>
+    <tableColumn id="7" name="Column8" headerRowDxfId="107" dataDxfId="106"/>
+    <tableColumn id="9" name="Column10" headerRowDxfId="105" dataDxfId="104"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4843,7 +3716,7 @@
         <v>24</v>
       </c>
       <c r="E19" s="25" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="F19" s="25" t="s">
         <v>12</v>
@@ -4878,7 +3751,7 @@
         <v>23</v>
       </c>
       <c r="E20" s="25" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="F20" s="25" t="s">
         <v>16</v>
@@ -4913,7 +3786,7 @@
         <v>25</v>
       </c>
       <c r="E21" s="25" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="F21" s="25" t="s">
         <v>18</v>
@@ -4948,7 +3821,7 @@
         <v>26</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="F22" s="25" t="s">
         <v>19</v>
@@ -5237,7 +4110,7 @@
         <v>51</v>
       </c>
       <c r="H30" s="21" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="I30" s="23" t="s">
         <v>15</v>
@@ -5893,7 +4766,7 @@
         <v>97</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F49" s="25" t="s">
         <v>98</v>
@@ -5928,7 +4801,7 @@
         <v>100</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F50" s="25" t="s">
         <v>101</v>
@@ -6068,7 +4941,7 @@
         <v>109</v>
       </c>
       <c r="E54" s="21" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F54" s="25" t="s">
         <v>111</v>
@@ -6103,7 +4976,7 @@
         <v>113</v>
       </c>
       <c r="E55" s="21" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F55" s="25" t="s">
         <v>114</v>
@@ -6243,7 +5116,7 @@
         <v>123</v>
       </c>
       <c r="E59" s="21" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F59" s="25" t="s">
         <v>124</v>
@@ -6278,7 +5151,7 @@
         <v>125</v>
       </c>
       <c r="E60" s="21" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F60" s="25" t="s">
         <v>126</v>
@@ -6376,8 +5249,8 @@
       <c r="B63" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="C63" s="12" t="s">
-        <v>137</v>
+      <c r="C63" s="20" t="s">
+        <v>136</v>
       </c>
       <c r="D63" s="13" t="s">
         <v>131</v>
@@ -6414,7 +5287,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{EDFDC9AB-9D9E-41E3-BC76-B8D67636F0EA}">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{EDFDC9AB-9D9E-41E3-BC76-B8D67636F0EA}">
             <xm:f>Support!$A$14</xm:f>
             <x14:dxf>
               <font>
@@ -6427,7 +5300,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{0E0E4D6F-12C1-4A01-8819-438A825BEC2D}">
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{0E0E4D6F-12C1-4A01-8819-438A825BEC2D}">
             <xm:f>Support!$A$13</xm:f>
             <x14:dxf>
               <font>
@@ -6443,7 +5316,7 @@
           <xm:sqref>C2:C63</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{E9C2B272-84B1-4809-B303-CE13207E6AB0}">
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{E9C2B272-84B1-4809-B303-CE13207E6AB0}">
             <xm:f>Support!$A$4</xm:f>
             <x14:dxf>
               <font>
@@ -6456,7 +5329,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="10" operator="equal" id="{E67A97B1-A6AA-4AEA-841E-887676001F2D}">
+          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{E67A97B1-A6AA-4AEA-841E-887676001F2D}">
             <xm:f>Support!$A$5</xm:f>
             <x14:dxf>
               <font>
@@ -6470,51 +5343,6 @@
             </x14:dxf>
           </x14:cfRule>
           <xm:sqref>I2:I63</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{45F6DB1C-4FF9-49E6-9475-597C87185476}">
-            <xm:f>Support!$A$17</xm:f>
-            <x14:dxf>
-              <font>
-                <color auto="1"/>
-              </font>
-              <fill>
-                <patternFill>
-                  <bgColor theme="3" tint="0.59996337778862885"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{C74CA95C-7727-418A-BE78-990F3D7CE068}">
-            <xm:f>Support!$A$18</xm:f>
-            <x14:dxf>
-              <font>
-                <color auto="1"/>
-              </font>
-              <fill>
-                <patternFill>
-                  <bgColor theme="7" tint="0.59996337778862885"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>B2:B63</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{3EE337D8-8BAD-4B99-8E46-C9C511026EE5}">
-            <xm:f>Support!$A$19</xm:f>
-            <x14:dxf>
-              <font>
-                <color auto="1"/>
-              </font>
-              <fill>
-                <patternFill>
-                  <bgColor theme="4" tint="0.59996337778862885"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>B63</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="cellIs" priority="3" operator="equal" id="{9540FE2F-D658-42C7-87B5-25E1482BD07B}">
@@ -6557,6 +5385,48 @@
             </x14:dxf>
           </x14:cfRule>
           <xm:sqref>J2:J63</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="8" id="{C74CA95C-7727-418A-BE78-990F3D7CE068}">
+            <xm:f>$B2=+Support!$A$18</xm:f>
+            <x14:dxf>
+              <font>
+                <color auto="1"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor theme="7" tint="0.79998168889431442"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="expression" priority="9" id="{45F6DB1C-4FF9-49E6-9475-597C87185476}">
+            <xm:f>$B2=Support!$A$17</xm:f>
+            <x14:dxf>
+              <font>
+                <color auto="1"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor theme="3" tint="0.79998168889431442"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="expression" priority="10" id="{3EE337D8-8BAD-4B99-8E46-C9C511026EE5}">
+            <xm:f>$B1048517=Support!$A$19</xm:f>
+            <x14:dxf>
+              <font>
+                <color auto="1"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor theme="4" tint="0.79998168889431442"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>A2:K63</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>